<commit_message>
chore: bundle reference docs + counter increment
- Pricelist_WorkBook_updated.xlsx (source for apply_pricebook_delta.py)
- Recuperator_Offer_Primary.docx (Viraj reference offer)
- USK Exports_ Recuperator_19.08.2025.xlsx (vendor BOM reference)
- Recuperator_Excel.xlsx + quote_counter.txt (working-state refresh)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Recuperator_Excel.xlsx
+++ b/Recuperator_Excel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RUPA\Downloads\offer_generator_structure\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{155DBFD4-4CB8-4C77-91C0-A7D7A6F570BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFB507D9-A60B-46FD-B2E2-1FB1FDD11D4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="95">
   <si>
     <t>Recuperator Calculation</t>
   </si>
@@ -391,6 +391,9 @@
   </si>
   <si>
     <t>NG</t>
+  </si>
+  <si>
+    <t>Total flue gas flow</t>
   </si>
 </sst>
 </file>
@@ -703,15 +706,15 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="10" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -949,7 +952,7 @@
     </row>
     <row r="2" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="3"/>
-      <c r="C2" s="49" t="s">
+      <c r="C2" s="46" t="s">
         <v>0</v>
       </c>
       <c r="D2" s="47"/>
@@ -967,13 +970,12 @@
     </row>
     <row r="3" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="3"/>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="48" t="s">
         <v>3</v>
       </c>
       <c r="D3" s="47"/>
       <c r="E3" s="8">
-        <f>E9+I7</f>
-        <v>1900</v>
+        <v>40000</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>4</v>
@@ -992,13 +994,13 @@
       <c r="B4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="48" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="47"/>
       <c r="E4" s="11">
         <f>E3*1.2</f>
-        <v>2280</v>
+        <v>48000</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>9</v>
@@ -1012,7 +1014,7 @@
     </row>
     <row r="5" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="3"/>
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="48" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="47"/>
@@ -1035,12 +1037,12 @@
     </row>
     <row r="6" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="48" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="47"/>
       <c r="E6" s="12">
-        <v>800</v>
+        <v>750</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>16</v>
@@ -1058,13 +1060,13 @@
     </row>
     <row r="7" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
-      <c r="C7" s="48" t="s">
+      <c r="C7" s="49" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="47"/>
       <c r="E7" s="13">
         <f>E6-(E13/(E4*E5))</f>
-        <v>438.96739130434776</v>
+        <v>496.28804347826087</v>
       </c>
       <c r="F7" s="14" t="s">
         <v>19</v>
@@ -1082,7 +1084,7 @@
     </row>
     <row r="8" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3"/>
-      <c r="C8" s="46" t="s">
+      <c r="C8" s="48" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="47"/>
@@ -1105,12 +1107,12 @@
     </row>
     <row r="9" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="3"/>
-      <c r="C9" s="46" t="s">
+      <c r="C9" s="48" t="s">
         <v>25</v>
       </c>
       <c r="D9" s="47"/>
       <c r="E9" s="15">
-        <v>1750</v>
+        <v>30000</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>4</v>
@@ -1128,7 +1130,7 @@
     </row>
     <row r="10" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="3"/>
-      <c r="C10" s="46" t="s">
+      <c r="C10" s="48" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="47"/>
@@ -1142,12 +1144,12 @@
     </row>
     <row r="11" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3"/>
-      <c r="C11" s="46" t="s">
+      <c r="C11" s="48" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="47"/>
       <c r="E11" s="17">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>30</v>
@@ -1157,7 +1159,7 @@
     </row>
     <row r="12" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="3"/>
-      <c r="C12" s="46" t="s">
+      <c r="C12" s="48" t="s">
         <v>31</v>
       </c>
       <c r="D12" s="47"/>
@@ -1173,13 +1175,13 @@
     </row>
     <row r="13" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="3"/>
-      <c r="C13" s="48" t="s">
+      <c r="C13" s="49" t="s">
         <v>32</v>
       </c>
       <c r="D13" s="47"/>
       <c r="E13" s="18">
         <f>(E9*1.2)*E12*(E11-E10)</f>
-        <v>189325.50000000003</v>
+        <v>2800980</v>
       </c>
       <c r="F13" s="14" t="s">
         <v>33</v>
@@ -1191,29 +1193,32 @@
       <c r="B14" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="46" t="s">
+      <c r="C14" s="48" t="s">
         <v>35</v>
       </c>
       <c r="D14" s="47"/>
       <c r="E14" s="20">
         <f>(((E6-E11)-(E7-E10))/(LN((E6-E11)/(E7-E10))))*0.9</f>
-        <v>361.78238934546329</v>
+        <v>386.92455827388829</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>36</v>
       </c>
       <c r="H14" s="1"/>
       <c r="I14" s="2"/>
+      <c r="J14" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="15" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="3"/>
-      <c r="C15" s="48" t="s">
+      <c r="C15" s="49" t="s">
         <v>37</v>
       </c>
       <c r="D15" s="47"/>
       <c r="E15" s="21">
         <f>(E13/(E14*E8))</f>
-        <v>17.443773345124928</v>
+        <v>241.30285349814881</v>
       </c>
       <c r="F15" s="14" t="s">
         <v>38</v>
@@ -1223,7 +1228,7 @@
     </row>
     <row r="16" spans="2:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="3"/>
-      <c r="C16" s="46" t="s">
+      <c r="C16" s="48" t="s">
         <v>39</v>
       </c>
       <c r="D16" s="47"/>
@@ -1239,7 +1244,7 @@
     </row>
     <row r="17" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="3"/>
-      <c r="C17" s="46" t="s">
+      <c r="C17" s="48" t="s">
         <v>41</v>
       </c>
       <c r="D17" s="47"/>
@@ -1270,13 +1275,13 @@
     </row>
     <row r="19" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="3"/>
-      <c r="C19" s="48" t="s">
+      <c r="C19" s="49" t="s">
         <v>43</v>
       </c>
       <c r="D19" s="47"/>
       <c r="E19" s="23">
         <f>E15/(3.14*(E23/1000)*(E24+0.1))</f>
-        <v>157.55812217186025</v>
+        <v>1243.0131100435756</v>
       </c>
       <c r="F19" s="14" t="s">
         <v>44</v>
@@ -1286,7 +1291,7 @@
     </row>
     <row r="20" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="3"/>
-      <c r="C20" s="46" t="s">
+      <c r="C20" s="48" t="s">
         <v>45</v>
       </c>
       <c r="D20" s="47"/>
@@ -1301,7 +1306,7 @@
     </row>
     <row r="21" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="3"/>
-      <c r="C21" s="46" t="s">
+      <c r="C21" s="48" t="s">
         <v>46</v>
       </c>
       <c r="D21" s="47"/>
@@ -1331,7 +1336,7 @@
     </row>
     <row r="23" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="3"/>
-      <c r="C23" s="46" t="s">
+      <c r="C23" s="48" t="s">
         <v>48</v>
       </c>
       <c r="D23" s="47"/>
@@ -1346,13 +1351,12 @@
     </row>
     <row r="24" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="3"/>
-      <c r="C24" s="46" t="s">
+      <c r="C24" s="48" t="s">
         <v>49</v>
       </c>
       <c r="D24" s="47"/>
       <c r="E24" s="26">
-        <f>0.55+0.08</f>
-        <v>0.63</v>
+        <v>1.18</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>50</v>
@@ -1377,7 +1381,7 @@
     </row>
     <row r="26" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="3"/>
-      <c r="C26" s="46" t="s">
+      <c r="C26" s="48" t="s">
         <v>52</v>
       </c>
       <c r="D26" s="47"/>
@@ -1392,13 +1396,13 @@
     </row>
     <row r="27" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="3"/>
-      <c r="C27" s="46" t="s">
+      <c r="C27" s="48" t="s">
         <v>54</v>
       </c>
       <c r="D27" s="47"/>
       <c r="E27" s="20">
         <f>E26*E24</f>
-        <v>1.9908000000000001</v>
+        <v>3.7288000000000001</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>55</v>
@@ -1408,13 +1412,13 @@
     </row>
     <row r="28" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="3"/>
-      <c r="C28" s="46" t="s">
+      <c r="C28" s="48" t="s">
         <v>56</v>
       </c>
       <c r="D28" s="47"/>
       <c r="E28" s="20">
         <f>(E27*(E20*(E21/2)))</f>
-        <v>167.22720000000001</v>
+        <v>313.2192</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>55</v>
@@ -1435,7 +1439,7 @@
     </row>
     <row r="30" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="3"/>
-      <c r="C30" s="46" t="s">
+      <c r="C30" s="48" t="s">
         <v>48</v>
       </c>
       <c r="D30" s="47"/>
@@ -1451,13 +1455,13 @@
     </row>
     <row r="31" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="3"/>
-      <c r="C31" s="46" t="s">
+      <c r="C31" s="48" t="s">
         <v>49</v>
       </c>
       <c r="D31" s="47"/>
       <c r="E31" s="26">
         <f t="shared" si="0"/>
-        <v>0.63</v>
+        <v>1.18</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>50</v>
@@ -1483,7 +1487,7 @@
     </row>
     <row r="33" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="3"/>
-      <c r="C33" s="46" t="s">
+      <c r="C33" s="48" t="s">
         <v>52</v>
       </c>
       <c r="D33" s="47"/>
@@ -1499,13 +1503,13 @@
     </row>
     <row r="34" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="3"/>
-      <c r="C34" s="46" t="s">
+      <c r="C34" s="48" t="s">
         <v>54</v>
       </c>
       <c r="D34" s="47"/>
       <c r="E34" s="20">
         <f>E33*E31</f>
-        <v>1.9908000000000001</v>
+        <v>3.7288000000000001</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>55</v>
@@ -1515,13 +1519,13 @@
     </row>
     <row r="35" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="3"/>
-      <c r="C35" s="46" t="s">
+      <c r="C35" s="48" t="s">
         <v>58</v>
       </c>
       <c r="D35" s="47"/>
       <c r="E35" s="20">
         <f>((E34*(E20*(E21/2))))</f>
-        <v>167.22720000000001</v>
+        <v>313.2192</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>55</v>
@@ -1531,7 +1535,7 @@
     </row>
     <row r="36" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="3"/>
-      <c r="C36" s="48" t="s">
+      <c r="C36" s="49" t="s">
         <v>59</v>
       </c>
       <c r="D36" s="47"/>
@@ -1542,7 +1546,7 @@
     </row>
     <row r="37" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="3"/>
-      <c r="C37" s="46" t="s">
+      <c r="C37" s="48" t="s">
         <v>60</v>
       </c>
       <c r="D37" s="47"/>
@@ -1557,7 +1561,7 @@
     </row>
     <row r="38" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="3"/>
-      <c r="C38" s="46" t="s">
+      <c r="C38" s="48" t="s">
         <v>62</v>
       </c>
       <c r="D38" s="47"/>
@@ -1573,7 +1577,7 @@
     </row>
     <row r="39" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3"/>
-      <c r="C39" s="46" t="s">
+      <c r="C39" s="48" t="s">
         <v>63</v>
       </c>
       <c r="D39" s="47"/>
@@ -1588,7 +1592,7 @@
     </row>
     <row r="40" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3"/>
-      <c r="C40" s="46" t="s">
+      <c r="C40" s="48" t="s">
         <v>64</v>
       </c>
       <c r="D40" s="47"/>
@@ -1597,20 +1601,20 @@
       </c>
       <c r="F40" s="11">
         <f>E28*F37+E35*F38</f>
-        <v>73579.968000000008</v>
+        <v>137816.448</v>
       </c>
       <c r="H40" s="1"/>
       <c r="I40" s="2"/>
     </row>
     <row r="41" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3"/>
-      <c r="C41" s="46" t="s">
+      <c r="C41" s="48" t="s">
         <v>65</v>
       </c>
       <c r="D41" s="47"/>
       <c r="E41" s="28">
         <f>((((2*E16)+100)*(E24*1000)*5)*(8650/1000000000)*2)</f>
-        <v>81.317438999999979</v>
+        <v>152.30885399999997</v>
       </c>
       <c r="F41" s="29" t="s">
         <v>55</v>
@@ -1740,7 +1744,7 @@
       </c>
       <c r="F49" s="32">
         <f>(E42+E41+E43+E44+E45+E46+E47)*F39</f>
-        <v>155978.69500236001</v>
+        <v>160238.17990235996</v>
       </c>
       <c r="H49" s="1"/>
       <c r="I49" s="2"/>
@@ -1820,7 +1824,7 @@
       </c>
       <c r="F54" s="32">
         <f>F40+F48+F49+F50+F51+F52+F53</f>
-        <v>312408.66300236003</v>
+        <v>380904.62790235993</v>
       </c>
       <c r="H54" s="1"/>
       <c r="I54" s="2"/>
@@ -1829,7 +1833,7 @@
       <c r="B55" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="C55" s="46" t="s">
+      <c r="C55" s="48" t="s">
         <v>82</v>
       </c>
       <c r="D55" s="47"/>
@@ -1863,7 +1867,7 @@
     </row>
     <row r="57" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="3"/>
-      <c r="C57" s="46" t="s">
+      <c r="C57" s="48" t="s">
         <v>85</v>
       </c>
       <c r="D57" s="47"/>
@@ -1903,7 +1907,7 @@
       </c>
       <c r="F59" s="32">
         <f>SUM(F54:F58)</f>
-        <v>368484.66300236003</v>
+        <v>436980.62790235993</v>
       </c>
       <c r="H59" s="1"/>
       <c r="I59" s="2"/>
@@ -1920,7 +1924,7 @@
       </c>
       <c r="F60" s="34">
         <f>F59*D60</f>
-        <v>663272.39340424805</v>
+        <v>786565.13022424793</v>
       </c>
       <c r="H60" s="1"/>
       <c r="I60" s="2"/>
@@ -1933,7 +1937,7 @@
       </c>
       <c r="F61" s="35">
         <f>F60</f>
-        <v>663272.39340424805</v>
+        <v>786565.13022424793</v>
       </c>
       <c r="H61" s="1"/>
       <c r="I61" s="2"/>
@@ -1950,7 +1954,7 @@
       </c>
       <c r="F62" s="39">
         <f>F61*D62</f>
-        <v>66327.239340424814</v>
+        <v>78656.513022424799</v>
       </c>
       <c r="H62" s="1"/>
       <c r="I62" s="2"/>
@@ -1967,7 +1971,7 @@
       </c>
       <c r="F63" s="39">
         <f>F61*D63</f>
-        <v>66327.239340424814</v>
+        <v>78656.513022424799</v>
       </c>
       <c r="H63" s="1"/>
       <c r="I63" s="2"/>
@@ -1982,7 +1986,7 @@
       </c>
       <c r="F64" s="43">
         <f>SUM(F61:F63)</f>
-        <v>795926.8720850976</v>
+        <v>943878.15626909747</v>
       </c>
       <c r="H64" s="1"/>
       <c r="I64" s="2"/>
@@ -5731,31 +5735,6 @@
     </row>
   </sheetData>
   <mergeCells count="37">
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="C26:D26"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C30:D30"/>
     <mergeCell ref="C31:D31"/>
     <mergeCell ref="C33:D33"/>
     <mergeCell ref="C34:D34"/>
@@ -5768,6 +5747,31 @@
     <mergeCell ref="C39:D39"/>
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="C30:D30"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>